<commit_message>
✨ feat: finished nomaddocs templates
</commit_message>
<xml_diff>
--- a/apps/excel-service/templates/NomadDocs/Cash Receipt Order.xlsx
+++ b/apps/excel-service/templates/NomadDocs/Cash Receipt Order.xlsx
@@ -1,46 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="18375"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="TDSheet" sheetId="1" r:id="rId1"/>
+    <sheet name="TDSheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
-    <t>- - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - л и н и я о т р е з а - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - -</t>
+    <t xml:space="preserve">- - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - л и н и я о т р е з а - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - - -</t>
   </si>
   <si>
-    <t>Приложение 1
+    <t xml:space="preserve">Приложение 1
 к приказу Министра финансов Республики Казахстан
 от 20 декабря 2012 года № 562</t>
   </si>
   <si>
-    <t>Форма КО-1</t>
+    <t xml:space="preserve">Форма КО-1</t>
   </si>
   <si>
-    <t>Организация (индивидуальный предприниматель)</t>
+    <t xml:space="preserve">Организация (индивидуальный предприниматель)</t>
   </si>
   <si>
     <t xml:space="preserve">Индивидуальный предприниматель                            ИП «NomadDocs»                                                              Жалтырбаев Әділет Ғалымұлы </t>
@@ -49,65 +38,37 @@
     <t>КВИТАНЦИЯ</t>
   </si>
   <si>
-    <t>к приходному кассовому ордеру</t>
+    <t xml:space="preserve">к приходному кассовому ордеру</t>
   </si>
   <si>
     <t>№</t>
   </si>
   <si>
-    <t>0081</t>
+    <t>{enumeration}</t>
   </si>
   <si>
-    <t>Принято от:</t>
+    <t xml:space="preserve">Принято от:</t>
   </si>
   <si>
-    <t>Темирбеков К.М.</t>
+    <t>{customer.fullnameClient}</t>
   </si>
   <si>
-    <t xml:space="preserve"> ТОО «Tranco Express»                                                                                                                                                                              индекс: 100601, РК, область Ұлытау, город сатпаев, Массив Промзона, строениие 169</t>
+    <t xml:space="preserve">{organization.organization}, {organization.address}</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Основание: Договор                </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-        <charset val="204"/>
-      </rPr>
-      <t>№0081</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="204"/>
-      </rPr>
-      <t>от  24.06.2026г</t>
-    </r>
+    <t xml:space="preserve">Основание: Договор               №{enumeration}               от  {documentDate.0}г </t>
   </si>
   <si>
-    <t xml:space="preserve">за проживание:  с 24.06.2026г- 26.06.2026г   </t>
+    <t xml:space="preserve">за проживание:  с  {documentDate.0}г - {documentDate.1}г</t>
   </si>
   <si>
     <t>Сумма</t>
   </si>
   <si>
-    <t xml:space="preserve">  40 00 тенге  00 тиын</t>
+    <t xml:space="preserve">  {totalPrice}  тенге  00 тиын</t>
   </si>
   <si>
-    <t>Сорок тысяч 00 тиын</t>
+    <t xml:space="preserve">{totalPriceWords} 00 тиын</t>
   </si>
   <si>
     <t>прописью</t>
@@ -128,7 +89,7 @@
     <t>подпись</t>
   </si>
   <si>
-    <t>расшифровка подписи</t>
+    <t xml:space="preserve">расшифровка подписи</t>
   </si>
   <si>
     <t>Кассир</t>
@@ -137,247 +98,188 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="167" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
-  <fonts count="33">
+  <fonts count="28">
     <font>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
+      <sz val="8.000000"/>
+      <color indexed="64"/>
       <name val="Arial"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="6"/>
-      <color theme="1"/>
+      <u/>
+      <sz val="11.000000"/>
+      <color indexed="4"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="7"/>
-      <color theme="1"/>
+      <u/>
+      <sz val="11.000000"/>
+      <color indexed="20"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="8"/>
-      <color theme="1"/>
+      <sz val="11.000000"/>
+      <color indexed="2"/>
       <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Arial"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="9"/>
-      <color theme="1"/>
+      <sz val="18.000000"/>
+      <color theme="3"/>
       <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8"/>
-      <name val="Arial"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="204"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <i/>
-      <sz val="6"/>
-      <color theme="1"/>
+      <sz val="11.000000"/>
+      <color rgb="FF7F7F7F"/>
       <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="18"/>
+      <sz val="15.000000"/>
       <color theme="3"/>
       <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="15"/>
+      <sz val="13.000000"/>
       <color theme="3"/>
       <name val="Arial"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="13"/>
+      <sz val="11.000000"/>
       <color theme="3"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="3"/>
+      <sz val="11.000000"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Arial"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <sz val="11.000000"/>
+      <color rgb="FFFA7D00"/>
       <name val="Arial"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="11.000000"/>
+      <color indexed="65"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
       <color rgb="FFFA7D00"/>
       <name val="Arial"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="11.000000"/>
+      <color theme="1"/>
       <name val="Arial"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <sz val="11.000000"/>
+      <color rgb="FF006100"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
+      <color rgb="FF9C0006"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
+      <color rgb="FF9C6500"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8.000000"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="6.000000"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="7.000000"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.000000"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="8.000000"/>
+      <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="9.000000"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
+      <b/>
+      <sz val="8.000000"/>
       <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <i/>
+      <sz val="6.000000"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Arial"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <charset val="204"/>
     </font>
   </fonts>
   <fills count="33">
@@ -389,207 +291,167 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
+        <fgColor indexed="26"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
+        <fgColor indexed="47"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="4" tint="0.79998168889431398"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="4" tint="0.59999389629810496"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="4" tint="0.39997558519241899"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="5" tint="0.79998168889431398"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="5" tint="0.59999389629810496"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="5" tint="0.39997558519241899"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="6" tint="0.79998168889431398"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="6" tint="0.59999389629810496"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="6" tint="0.39997558519241899"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="7" tint="0.79998168889431398"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="7" tint="0.59999389629810496"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="7" tint="0.39997558519241899"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="8" tint="0.79998168889431398"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="8" tint="0.59999389629810496"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="8" tint="0.39997558519241899"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="9" tint="0.79998168889431398"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="9" tint="0.59999389629810496"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="9" tint="0.39997558519241899"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="10">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
@@ -604,25 +466,25 @@
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
       <bottom style="medium">
         <color theme="4"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
       <bottom style="medium">
         <color theme="4" tint="0.499984740745262"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
@@ -637,7 +499,7 @@
       <bottom style="thin">
         <color rgb="FF7F7F7F"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
@@ -652,7 +514,7 @@
       <bottom style="thin">
         <color rgb="FF3F3F3F"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="double">
@@ -667,240 +529,243 @@
       <bottom style="double">
         <color rgb="FF3F3F3F"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
       <bottom style="double">
         <color rgb="FFFF8001"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="none"/>
+      <right style="none"/>
       <top style="thin">
         <color theme="4"/>
       </top>
       <bottom style="double">
         <color theme="4"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="164" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="165" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="166" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="167" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" applyNumberFormat="0" applyFont="0" applyFill="1" applyBorder="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="6" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="7" fillId="0" borderId="2" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="8" fillId="0" borderId="2" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="9" fillId="0" borderId="3" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="9" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="10" fillId="3" borderId="4" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="11" fillId="4" borderId="5" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="12" fillId="4" borderId="4" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="13" fillId="5" borderId="6" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="14" fillId="0" borderId="7" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="15" fillId="0" borderId="8" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="16" fillId="6" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="17" fillId="7" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="18" fillId="8" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="19" fillId="9" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="10" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="11" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="19" fillId="12" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="19" fillId="13" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="14" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="15" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="19" fillId="16" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="19" fillId="17" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="18" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="19" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="19" fillId="20" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="19" fillId="21" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="22" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="23" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="19" fillId="24" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="19" fillId="25" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="26" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="27" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="19" fillId="28" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="19" fillId="29" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="30" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="1" fillId="31" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf fontId="19" fillId="32" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="23">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+  <cellXfs count="21">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="20" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="21" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" vertical="center"/>
+    </xf>
+    <xf fontId="22" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="20" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="20" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="23" fillId="0" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="24" fillId="0" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="25" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="23" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="26" fillId="0" borderId="9" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="23" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="20" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="20" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="20" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="23" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="27" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf fontId="23" fillId="0" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="23" fillId="0" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="20" fillId="0" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="20" fillId="0" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -957,47 +822,30 @@
   </cellStyles>
   <dxfs count="17">
     <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79998168889431398"/>
+          <bgColor theme="4" tint="0.79998168889431398"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79998168889431398"/>
+          <bgColor theme="4" tint="0.79998168889431398"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="double">
-          <color theme="4"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
+        <b/>
         <color theme="0"/>
       </font>
       <fill>
@@ -1006,6 +854,27 @@
           <bgColor theme="4"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <left/>
+        <right/>
+        <top style="double">
+          <color theme="4"/>
+        </top>
+        <bottom/>
+        <diagonal/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1024,38 +893,115 @@
         <bottom style="thin">
           <color theme="4"/>
         </bottom>
+        <diagonal/>
         <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
+          <color theme="4" tint="0.39997558519241899"/>
         </horizontal>
       </border>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79998168889431398"/>
+          <bgColor theme="4" tint="0.79998168889431398"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431398"/>
+          <bgColor theme="4" tint="0.79998168889431398"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
       <border>
+        <left/>
+        <right/>
+        <top/>
         <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
+          <color theme="4" tint="0.39997558519241899"/>
         </bottom>
+        <diagonal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79998168889431398"/>
+          <bgColor theme="4" tint="0.79998168889431398"/>
         </patternFill>
       </fill>
       <border>
+        <left/>
+        <right/>
+        <top/>
         <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
+          <color theme="4" tint="0.39997558519241899"/>
         </bottom>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431398"/>
+          <bgColor theme="4" tint="0.79998168889431398"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241899"/>
+        </bottom>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431398"/>
+          <bgColor theme="4" tint="0.79998168889431398"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241899"/>
+        </bottom>
+        <diagonal/>
       </border>
     </dxf>
     <dxf>
@@ -1065,116 +1011,57 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79998168889431398"/>
+          <bgColor theme="4" tint="0.79998168889431398"/>
         </patternFill>
       </fill>
       <border>
+        <left/>
+        <right/>
         <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
+          <color theme="4" tint="0.39997558519241899"/>
         </top>
         <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
+          <color theme="4" tint="0.39997558519241899"/>
         </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
+        <diagonal/>
       </border>
     </dxf>
   </dxfs>
-  <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+  <tableStyles count="2" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
+      <tableStyleElement type="firstColumn" size="1" dxfId="0"/>
+      <tableStyleElement type="firstColumnStripe" size="1" dxfId="1"/>
+      <tableStyleElement type="firstRowStripe" size="1" dxfId="2"/>
+      <tableStyleElement type="headerRow" size="1" dxfId="3"/>
+      <tableStyleElement type="lastColumn" size="1" dxfId="4"/>
+      <tableStyleElement type="totalRow" size="1" dxfId="5"/>
+      <tableStyleElement type="wholeTable" size="1" dxfId="6"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
+      <tableStyleElement type="firstColumnStripe" size="1" dxfId="7"/>
+      <tableStyleElement type="firstRowStripe" size="1" dxfId="8"/>
+      <tableStyleElement type="firstRowSubheading" size="1" dxfId="9"/>
+      <tableStyleElement type="firstSubtotalRow" size="1" dxfId="10"/>
+      <tableStyleElement type="headerRow" size="1" dxfId="11"/>
+      <tableStyleElement type="pageFieldLabels" size="1" dxfId="12"/>
+      <tableStyleElement type="pageFieldValues" size="1" dxfId="13"/>
+      <tableStyleElement type="secondRowSubheading" size="1" dxfId="14"/>
+      <tableStyleElement type="secondSubtotalRow" size="1" dxfId="15"/>
+      <tableStyleElement type="totalRow" size="1" dxfId="16"/>
     </tableStyle>
   </tableStyles>
-  <colors>
-    <mruColors>
-      <color rgb="00000000"/>
-    </mruColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1183,8 +1070,291 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1241,7 +1411,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1267,7 +1437,7 @@
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1344,7 +1514,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1379,24 +1549,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I1000"/>
   <sheetFormatPr defaultColWidth="16.7777777777778" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="4.66666666666667" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="1.44444444444444" customWidth="1"/>
-    <col min="3" max="3" width="8.66666666666667" customWidth="1"/>
-    <col min="4" max="5" width="1.44444444444444" customWidth="1"/>
-    <col min="6" max="6" width="8.33333333333333" customWidth="1"/>
-    <col min="7" max="7" width="1.77777777777778" customWidth="1"/>
-    <col min="8" max="8" width="21.6666666666667" customWidth="1"/>
-    <col min="9" max="9" width="0.111111111111111" customWidth="1"/>
+    <col customWidth="1" hidden="1" min="1" max="1" width="4.6666666666666696"/>
+    <col customWidth="1" min="2" max="2" width="1.44444444444444"/>
+    <col customWidth="1" min="3" max="3" width="8.6666666666666696"/>
+    <col customWidth="1" min="4" max="5" width="1.44444444444444"/>
+    <col customWidth="1" min="6" max="6" width="8.3333333333333304"/>
+    <col customWidth="1" min="7" max="7" width="1.7777777777777799"/>
+    <col customWidth="1" min="8" max="8" width="21.6666666666667"/>
+    <col customWidth="1" min="9" max="9" width="0.11111111111111099"/>
   </cols>
   <sheetData>
-    <row r="1" ht="9.75" customHeight="1" spans="1:9">
+    <row r="1" ht="9.75" customHeight="1">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1407,7 +1577,7 @@
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
     </row>
-    <row r="2" ht="9.75" customHeight="1" spans="1:9">
+    <row r="2" ht="9.75" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1418,7 +1588,7 @@
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
     </row>
-    <row r="3" ht="9.75" customHeight="1" spans="1:9">
+    <row r="3" ht="9.75" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1429,7 +1599,7 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
     </row>
-    <row r="4" ht="9.75" customHeight="1" spans="1:9">
+    <row r="4" ht="9.75" customHeight="1">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -1440,7 +1610,7 @@
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
     </row>
-    <row r="5" ht="9.75" customHeight="1" spans="1:9">
+    <row r="5" ht="9.75" customHeight="1">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -1451,7 +1621,7 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
     </row>
-    <row r="6" ht="9.75" customHeight="1" spans="1:9">
+    <row r="6" ht="9.75" customHeight="1">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -1462,7 +1632,7 @@
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
     </row>
-    <row r="7" ht="9.75" customHeight="1" spans="1:3">
+    <row r="7" ht="9.75" customHeight="1">
       <c r="A7" s="1"/>
       <c r="B7" s="2" t="s">
         <v>0</v>
@@ -1471,13 +1641,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" ht="9.75" customHeight="1" spans="1:1">
+    <row r="8" ht="9.75" customHeight="1">
       <c r="A8" s="1"/>
     </row>
-    <row r="9" ht="9.75" customHeight="1" spans="1:1">
+    <row r="9" ht="9.75" customHeight="1">
       <c r="A9" s="1"/>
     </row>
-    <row r="10" ht="9.75" customHeight="1" spans="1:6">
+    <row r="10" ht="9.75" customHeight="1">
       <c r="A10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -1486,7 +1656,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" ht="9.75" customHeight="1" spans="1:9">
+    <row r="11" ht="9.75" customHeight="1">
       <c r="A11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -1496,14 +1666,14 @@
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
     </row>
-    <row r="12" ht="9.75" customHeight="1" spans="1:9">
+    <row r="12" ht="9.75" customHeight="1">
       <c r="A12" s="1"/>
       <c r="C12" s="5" t="s">
         <v>3</v>
       </c>
       <c r="I12" s="1"/>
     </row>
-    <row r="13" ht="36" customHeight="1" spans="1:9">
+    <row r="13" ht="36" customHeight="1">
       <c r="A13" s="1"/>
       <c r="C13" s="6" t="s">
         <v>4</v>
@@ -1515,7 +1685,7 @@
       <c r="H13" s="7"/>
       <c r="I13" s="1"/>
     </row>
-    <row r="14" ht="9.75" customHeight="1" spans="1:9">
+    <row r="14" ht="9.75" customHeight="1">
       <c r="A14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -1525,21 +1695,21 @@
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
     </row>
-    <row r="15" ht="11.25" customHeight="1" spans="1:9">
+    <row r="15" ht="11.25" customHeight="1">
       <c r="A15" s="1"/>
       <c r="C15" s="8" t="s">
         <v>5</v>
       </c>
       <c r="I15" s="1"/>
     </row>
-    <row r="16" ht="10.5" customHeight="1" spans="1:9">
+    <row r="16" ht="10.5" customHeight="1">
       <c r="A16" s="1"/>
       <c r="C16" s="9" t="s">
         <v>6</v>
       </c>
       <c r="I16" s="1"/>
     </row>
-    <row r="17" ht="10.5" customHeight="1" spans="1:9">
+    <row r="17" ht="10.5" customHeight="1">
       <c r="A17" s="1"/>
       <c r="C17" s="4" t="s">
         <v>7</v>
@@ -1553,7 +1723,7 @@
       <c r="H17" s="11"/>
       <c r="I17" s="1"/>
     </row>
-    <row r="18" ht="9.75" customHeight="1" spans="1:9">
+    <row r="18" ht="9.75" customHeight="1">
       <c r="A18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
@@ -1563,7 +1733,7 @@
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
     </row>
-    <row r="19" ht="18.75" customHeight="1" spans="1:9">
+    <row r="19" ht="18.75" customHeight="1">
       <c r="A19" s="1"/>
       <c r="C19" s="12" t="s">
         <v>9</v>
@@ -1573,18 +1743,18 @@
       </c>
       <c r="I19" s="1"/>
     </row>
-    <row r="20" ht="9.75" customHeight="1" spans="1:9">
+    <row r="20" ht="9.75" customHeight="1">
       <c r="A20" s="1"/>
       <c r="C20" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="I20" s="14"/>
-    </row>
-    <row r="21" ht="9.75" customHeight="1" spans="1:9">
+      <c r="I20" s="13"/>
+    </row>
+    <row r="21" ht="9.75" customHeight="1">
       <c r="A21" s="1"/>
-      <c r="I21" s="14"/>
-    </row>
-    <row r="22" ht="35.25" customHeight="1" spans="1:9">
+      <c r="I21" s="13"/>
+    </row>
+    <row r="22" ht="35.25" customHeight="1">
       <c r="A22" s="1"/>
       <c r="C22" s="7"/>
       <c r="D22" s="7"/>
@@ -1592,30 +1762,30 @@
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
       <c r="H22" s="7"/>
-      <c r="I22" s="14"/>
-    </row>
-    <row r="23" ht="53.25" customHeight="1" spans="1:9">
+      <c r="I22" s="13"/>
+    </row>
+    <row r="23" ht="53.25" customHeight="1">
       <c r="A23" s="1"/>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
-    </row>
-    <row r="24" ht="9.75" customHeight="1" spans="1:9">
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="13"/>
+    </row>
+    <row r="24" ht="9.75" customHeight="1">
       <c r="A24" s="1"/>
-      <c r="C24" s="15" t="s">
+      <c r="C24" s="12" t="s">
         <v>13</v>
       </c>
       <c r="I24" s="1"/>
     </row>
-    <row r="25" ht="9.75" customHeight="1" spans="1:9">
+    <row r="25" ht="9.75" customHeight="1">
       <c r="A25" s="1"/>
       <c r="I25" s="1"/>
     </row>
-    <row r="26" ht="9.75" customHeight="1" spans="1:9">
+    <row r="26" ht="9.75" customHeight="1">
       <c r="A26" s="1"/>
       <c r="C26" s="7"/>
       <c r="D26" s="7"/>
@@ -1625,7 +1795,7 @@
       <c r="H26" s="7"/>
       <c r="I26" s="1"/>
     </row>
-    <row r="27" ht="9.75" customHeight="1" spans="1:9">
+    <row r="27" ht="9.75" customHeight="1">
       <c r="A27" s="1"/>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
@@ -1635,24 +1805,24 @@
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
     </row>
-    <row r="28" ht="21" customHeight="1" spans="1:9">
+    <row r="28" ht="21" customHeight="1">
       <c r="A28" s="1"/>
       <c r="C28" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D28" s="16" t="s">
+      <c r="D28" s="5" t="s">
         <v>15</v>
       </c>
       <c r="I28" s="1"/>
     </row>
-    <row r="29" ht="9.75" customHeight="1" spans="1:9">
+    <row r="29" ht="9.75" customHeight="1">
       <c r="A29" s="1"/>
-      <c r="C29" s="17" t="s">
+      <c r="C29" s="15" t="s">
         <v>16</v>
       </c>
       <c r="I29" s="1"/>
     </row>
-    <row r="30" ht="9.75" customHeight="1" spans="1:9">
+    <row r="30" ht="9.75" customHeight="1">
       <c r="A30" s="1"/>
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
@@ -1662,10 +1832,10 @@
       <c r="H30" s="7"/>
       <c r="I30" s="1"/>
     </row>
-    <row r="31" ht="9.75" customHeight="1" spans="1:9">
+    <row r="31" ht="9.75" customHeight="1">
       <c r="A31" s="1"/>
       <c r="C31" s="1"/>
-      <c r="D31" s="18" t="s">
+      <c r="D31" s="16" t="s">
         <v>17</v>
       </c>
       <c r="E31" s="1"/>
@@ -1674,7 +1844,7 @@
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
     </row>
-    <row r="32" ht="10.5" customHeight="1" spans="1:9">
+    <row r="32" ht="10.5" customHeight="1">
       <c r="A32" s="1"/>
       <c r="C32" s="1" t="s">
         <v>18</v>
@@ -1682,7 +1852,7 @@
       <c r="D32" s="9"/>
       <c r="I32" s="1"/>
     </row>
-    <row r="33" ht="9.75" customHeight="1" spans="1:9">
+    <row r="33" ht="9.75" customHeight="1">
       <c r="A33" s="1"/>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
@@ -1692,7 +1862,7 @@
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
     </row>
-    <row r="34" ht="10.5" customHeight="1" spans="1:9">
+    <row r="34" ht="10.5" customHeight="1">
       <c r="A34" s="1"/>
       <c r="C34" s="11" t="s">
         <v>19</v>
@@ -1704,32 +1874,32 @@
       <c r="H34" s="11"/>
       <c r="I34" s="1"/>
     </row>
-    <row r="35" ht="25.5" customHeight="1" spans="1:9">
+    <row r="35" ht="25.5" customHeight="1">
       <c r="A35" s="1"/>
-      <c r="C35" s="19"/>
+      <c r="C35" s="17"/>
       <c r="D35" s="7"/>
       <c r="E35" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="F35" s="20" t="s">
+      <c r="F35" s="18" t="s">
         <v>21</v>
       </c>
       <c r="G35" s="7"/>
       <c r="H35" s="7"/>
       <c r="I35" s="1"/>
     </row>
-    <row r="36" ht="9.75" customHeight="1" spans="1:9">
+    <row r="36" ht="9.75" customHeight="1">
       <c r="A36" s="1"/>
-      <c r="C36" s="18" t="s">
+      <c r="C36" s="16" t="s">
         <v>22</v>
       </c>
       <c r="E36" s="1"/>
-      <c r="F36" s="18" t="s">
+      <c r="F36" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I36" s="1"/>
     </row>
-    <row r="37" ht="9.75" customHeight="1" spans="1:9">
+    <row r="37" ht="9.75" customHeight="1">
       <c r="A37" s="1"/>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
@@ -1739,43 +1909,43 @@
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
     </row>
-    <row r="38" ht="9.75" customHeight="1" spans="1:9">
+    <row r="38" ht="9.75" customHeight="1">
       <c r="A38" s="1"/>
       <c r="C38" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D38" s="21"/>
+      <c r="D38" s="19"/>
       <c r="E38" s="7"/>
       <c r="F38" s="7"/>
       <c r="G38" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H38" s="22"/>
+      <c r="H38" s="20"/>
       <c r="I38" s="1"/>
     </row>
-    <row r="39" ht="9.75" customHeight="1" spans="1:9">
+    <row r="39" ht="9.75" customHeight="1">
       <c r="A39" s="1"/>
       <c r="C39" s="1"/>
-      <c r="D39" s="18" t="s">
+      <c r="D39" s="16" t="s">
         <v>22</v>
       </c>
       <c r="G39" s="1"/>
-      <c r="H39" s="18" t="s">
+      <c r="H39" s="16" t="s">
         <v>23</v>
       </c>
       <c r="I39" s="1"/>
     </row>
-    <row r="40" ht="9.75" customHeight="1" spans="1:9">
+    <row r="40" ht="9.75" customHeight="1">
       <c r="A40" s="1"/>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
-      <c r="G40" s="18"/>
-      <c r="H40" s="18"/>
+      <c r="G40" s="16"/>
+      <c r="H40" s="16"/>
       <c r="I40" s="1"/>
     </row>
-    <row r="41" ht="9.75" customHeight="1" spans="1:9">
+    <row r="41" ht="9.75" customHeight="1">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -1786,7 +1956,7 @@
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
     </row>
-    <row r="42" ht="9.75" customHeight="1" spans="1:9">
+    <row r="42" ht="9.75" customHeight="1">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -1797,7 +1967,7 @@
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
     </row>
-    <row r="43" ht="9.75" customHeight="1" spans="1:9">
+    <row r="43" ht="9.75" customHeight="1">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -1808,7 +1978,7 @@
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
     </row>
-    <row r="44" ht="9.75" customHeight="1" spans="1:9">
+    <row r="44" ht="9.75" customHeight="1">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -1819,7 +1989,7 @@
       <c r="H44" s="1"/>
       <c r="I44" s="1"/>
     </row>
-    <row r="45" ht="9.75" customHeight="1" spans="1:9">
+    <row r="45" ht="9.75" customHeight="1">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -1830,7 +2000,7 @@
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
     </row>
-    <row r="46" ht="9.75" customHeight="1" spans="1:9">
+    <row r="46" ht="9.75" customHeight="1">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -1841,7 +2011,7 @@
       <c r="H46" s="1"/>
       <c r="I46" s="1"/>
     </row>
-    <row r="47" ht="9.75" customHeight="1" spans="1:9">
+    <row r="47" ht="9.75" customHeight="1">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -1852,7 +2022,7 @@
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
     </row>
-    <row r="48" ht="9.75" customHeight="1" spans="1:9">
+    <row r="48" ht="9.75" customHeight="1">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -1863,7 +2033,7 @@
       <c r="H48" s="1"/>
       <c r="I48" s="1"/>
     </row>
-    <row r="49" ht="9.75" customHeight="1" spans="1:9">
+    <row r="49" ht="9.75" customHeight="1">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -1874,7 +2044,7 @@
       <c r="H49" s="1"/>
       <c r="I49" s="1"/>
     </row>
-    <row r="50" ht="9.75" customHeight="1" spans="1:9">
+    <row r="50" ht="9.75" customHeight="1">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -1885,7 +2055,7 @@
       <c r="H50" s="1"/>
       <c r="I50" s="1"/>
     </row>
-    <row r="51" ht="9.75" customHeight="1" spans="1:9">
+    <row r="51" ht="9.75" customHeight="1">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
@@ -1896,7 +2066,7 @@
       <c r="H51" s="1"/>
       <c r="I51" s="1"/>
     </row>
-    <row r="52" ht="9.75" customHeight="1" spans="1:9">
+    <row r="52" ht="9.75" customHeight="1">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -1907,7 +2077,7 @@
       <c r="H52" s="1"/>
       <c r="I52" s="1"/>
     </row>
-    <row r="53" ht="9.75" customHeight="1" spans="1:9">
+    <row r="53" ht="9.75" customHeight="1">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -1918,7 +2088,7 @@
       <c r="H53" s="1"/>
       <c r="I53" s="1"/>
     </row>
-    <row r="54" ht="9.75" customHeight="1" spans="1:9">
+    <row r="54" ht="9.75" customHeight="1">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -1929,7 +2099,7 @@
       <c r="H54" s="1"/>
       <c r="I54" s="1"/>
     </row>
-    <row r="55" ht="9.75" customHeight="1" spans="1:9">
+    <row r="55" ht="9.75" customHeight="1">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -1940,7 +2110,7 @@
       <c r="H55" s="1"/>
       <c r="I55" s="1"/>
     </row>
-    <row r="56" ht="9.75" customHeight="1" spans="1:9">
+    <row r="56" ht="9.75" customHeight="1">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
@@ -1951,7 +2121,7 @@
       <c r="H56" s="1"/>
       <c r="I56" s="1"/>
     </row>
-    <row r="57" ht="9.75" customHeight="1" spans="1:9">
+    <row r="57" ht="9.75" customHeight="1">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
@@ -1962,7 +2132,7 @@
       <c r="H57" s="1"/>
       <c r="I57" s="1"/>
     </row>
-    <row r="58" ht="9.75" customHeight="1" spans="1:9">
+    <row r="58" ht="9.75" customHeight="1">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
@@ -1973,7 +2143,7 @@
       <c r="H58" s="1"/>
       <c r="I58" s="1"/>
     </row>
-    <row r="59" ht="9.75" customHeight="1" spans="1:9">
+    <row r="59" ht="9.75" customHeight="1">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
@@ -1984,7 +2154,7 @@
       <c r="H59" s="1"/>
       <c r="I59" s="1"/>
     </row>
-    <row r="60" ht="9.75" customHeight="1" spans="1:9">
+    <row r="60" ht="9.75" customHeight="1">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
@@ -1995,7 +2165,7 @@
       <c r="H60" s="1"/>
       <c r="I60" s="1"/>
     </row>
-    <row r="61" ht="9.75" customHeight="1" spans="1:9">
+    <row r="61" ht="9.75" customHeight="1">
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
@@ -2006,7 +2176,7 @@
       <c r="H61" s="1"/>
       <c r="I61" s="1"/>
     </row>
-    <row r="62" ht="9.75" customHeight="1" spans="1:9">
+    <row r="62" ht="9.75" customHeight="1">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
@@ -2017,7 +2187,7 @@
       <c r="H62" s="1"/>
       <c r="I62" s="1"/>
     </row>
-    <row r="63" ht="9.75" customHeight="1" spans="1:9">
+    <row r="63" ht="9.75" customHeight="1">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
@@ -2028,7 +2198,7 @@
       <c r="H63" s="1"/>
       <c r="I63" s="1"/>
     </row>
-    <row r="64" ht="9.75" customHeight="1" spans="1:9">
+    <row r="64" ht="9.75" customHeight="1">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
@@ -2039,7 +2209,7 @@
       <c r="H64" s="1"/>
       <c r="I64" s="1"/>
     </row>
-    <row r="65" ht="9.75" customHeight="1" spans="1:9">
+    <row r="65" ht="9.75" customHeight="1">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
@@ -2050,7 +2220,7 @@
       <c r="H65" s="1"/>
       <c r="I65" s="1"/>
     </row>
-    <row r="66" ht="9.75" customHeight="1" spans="1:9">
+    <row r="66" ht="9.75" customHeight="1">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
@@ -2061,7 +2231,7 @@
       <c r="H66" s="1"/>
       <c r="I66" s="1"/>
     </row>
-    <row r="67" ht="9.75" customHeight="1" spans="1:9">
+    <row r="67" ht="9.75" customHeight="1">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
@@ -2072,7 +2242,7 @@
       <c r="H67" s="1"/>
       <c r="I67" s="1"/>
     </row>
-    <row r="68" ht="9.75" customHeight="1" spans="1:9">
+    <row r="68" ht="9.75" customHeight="1">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
@@ -2083,7 +2253,7 @@
       <c r="H68" s="1"/>
       <c r="I68" s="1"/>
     </row>
-    <row r="69" ht="9.75" customHeight="1" spans="1:9">
+    <row r="69" ht="9.75" customHeight="1">
       <c r="A69" s="1"/>
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
@@ -2094,7 +2264,7 @@
       <c r="H69" s="1"/>
       <c r="I69" s="1"/>
     </row>
-    <row r="70" ht="9.75" customHeight="1" spans="1:9">
+    <row r="70" ht="9.75" customHeight="1">
       <c r="A70" s="1"/>
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
@@ -2105,7 +2275,7 @@
       <c r="H70" s="1"/>
       <c r="I70" s="1"/>
     </row>
-    <row r="71" ht="9.75" customHeight="1" spans="1:9">
+    <row r="71" ht="9.75" customHeight="1">
       <c r="A71" s="1"/>
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
@@ -2116,7 +2286,7 @@
       <c r="H71" s="1"/>
       <c r="I71" s="1"/>
     </row>
-    <row r="72" ht="9.75" customHeight="1" spans="1:9">
+    <row r="72" ht="9.75" customHeight="1">
       <c r="A72" s="1"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
@@ -2127,7 +2297,7 @@
       <c r="H72" s="1"/>
       <c r="I72" s="1"/>
     </row>
-    <row r="73" ht="9.75" customHeight="1" spans="1:9">
+    <row r="73" ht="9.75" customHeight="1">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
@@ -2138,7 +2308,7 @@
       <c r="H73" s="1"/>
       <c r="I73" s="1"/>
     </row>
-    <row r="74" ht="9.75" customHeight="1" spans="1:9">
+    <row r="74" ht="9.75" customHeight="1">
       <c r="A74" s="1"/>
       <c r="B74" s="1"/>
       <c r="C74" s="1"/>
@@ -2149,7 +2319,7 @@
       <c r="H74" s="1"/>
       <c r="I74" s="1"/>
     </row>
-    <row r="75" ht="9.75" customHeight="1" spans="1:9">
+    <row r="75" ht="9.75" customHeight="1">
       <c r="A75" s="1"/>
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
@@ -2160,7 +2330,7 @@
       <c r="H75" s="1"/>
       <c r="I75" s="1"/>
     </row>
-    <row r="76" ht="9.75" customHeight="1" spans="1:9">
+    <row r="76" ht="9.75" customHeight="1">
       <c r="A76" s="1"/>
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
@@ -2171,7 +2341,7 @@
       <c r="H76" s="1"/>
       <c r="I76" s="1"/>
     </row>
-    <row r="77" ht="9.75" customHeight="1" spans="1:9">
+    <row r="77" ht="9.75" customHeight="1">
       <c r="A77" s="1"/>
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
@@ -2182,7 +2352,7 @@
       <c r="H77" s="1"/>
       <c r="I77" s="1"/>
     </row>
-    <row r="78" ht="9.75" customHeight="1" spans="1:9">
+    <row r="78" ht="9.75" customHeight="1">
       <c r="A78" s="1"/>
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
@@ -2193,7 +2363,7 @@
       <c r="H78" s="1"/>
       <c r="I78" s="1"/>
     </row>
-    <row r="79" ht="9.75" customHeight="1" spans="1:9">
+    <row r="79" ht="9.75" customHeight="1">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
@@ -2204,7 +2374,7 @@
       <c r="H79" s="1"/>
       <c r="I79" s="1"/>
     </row>
-    <row r="80" ht="9.75" customHeight="1" spans="1:9">
+    <row r="80" ht="9.75" customHeight="1">
       <c r="A80" s="1"/>
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
@@ -2215,7 +2385,7 @@
       <c r="H80" s="1"/>
       <c r="I80" s="1"/>
     </row>
-    <row r="81" ht="9.75" customHeight="1" spans="1:9">
+    <row r="81" ht="9.75" customHeight="1">
       <c r="A81" s="1"/>
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
@@ -2226,7 +2396,7 @@
       <c r="H81" s="1"/>
       <c r="I81" s="1"/>
     </row>
-    <row r="82" ht="9.75" customHeight="1" spans="1:9">
+    <row r="82" ht="9.75" customHeight="1">
       <c r="A82" s="1"/>
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
@@ -2237,7 +2407,7 @@
       <c r="H82" s="1"/>
       <c r="I82" s="1"/>
     </row>
-    <row r="83" ht="9.75" customHeight="1" spans="1:9">
+    <row r="83" ht="9.75" customHeight="1">
       <c r="A83" s="1"/>
       <c r="B83" s="1"/>
       <c r="C83" s="1"/>
@@ -2248,7 +2418,7 @@
       <c r="H83" s="1"/>
       <c r="I83" s="1"/>
     </row>
-    <row r="84" ht="9.75" customHeight="1" spans="1:9">
+    <row r="84" ht="9.75" customHeight="1">
       <c r="A84" s="1"/>
       <c r="B84" s="1"/>
       <c r="C84" s="1"/>
@@ -2259,7 +2429,7 @@
       <c r="H84" s="1"/>
       <c r="I84" s="1"/>
     </row>
-    <row r="85" ht="9.75" customHeight="1" spans="1:9">
+    <row r="85" ht="9.75" customHeight="1">
       <c r="A85" s="1"/>
       <c r="B85" s="1"/>
       <c r="C85" s="1"/>
@@ -2270,7 +2440,7 @@
       <c r="H85" s="1"/>
       <c r="I85" s="1"/>
     </row>
-    <row r="86" ht="9.75" customHeight="1" spans="1:9">
+    <row r="86" ht="9.75" customHeight="1">
       <c r="A86" s="1"/>
       <c r="B86" s="1"/>
       <c r="C86" s="1"/>
@@ -2281,7 +2451,7 @@
       <c r="H86" s="1"/>
       <c r="I86" s="1"/>
     </row>
-    <row r="87" ht="9.75" customHeight="1" spans="1:9">
+    <row r="87" ht="9.75" customHeight="1">
       <c r="A87" s="1"/>
       <c r="B87" s="1"/>
       <c r="C87" s="1"/>
@@ -2292,7 +2462,7 @@
       <c r="H87" s="1"/>
       <c r="I87" s="1"/>
     </row>
-    <row r="88" ht="9.75" customHeight="1" spans="1:9">
+    <row r="88" ht="9.75" customHeight="1">
       <c r="A88" s="1"/>
       <c r="B88" s="1"/>
       <c r="C88" s="1"/>
@@ -2303,7 +2473,7 @@
       <c r="H88" s="1"/>
       <c r="I88" s="1"/>
     </row>
-    <row r="89" ht="9.75" customHeight="1" spans="1:9">
+    <row r="89" ht="9.75" customHeight="1">
       <c r="A89" s="1"/>
       <c r="B89" s="1"/>
       <c r="C89" s="1"/>
@@ -2314,7 +2484,7 @@
       <c r="H89" s="1"/>
       <c r="I89" s="1"/>
     </row>
-    <row r="90" ht="9.75" customHeight="1" spans="1:9">
+    <row r="90" ht="9.75" customHeight="1">
       <c r="A90" s="1"/>
       <c r="B90" s="1"/>
       <c r="C90" s="1"/>
@@ -2325,7 +2495,7 @@
       <c r="H90" s="1"/>
       <c r="I90" s="1"/>
     </row>
-    <row r="91" ht="9.75" customHeight="1" spans="1:9">
+    <row r="91" ht="9.75" customHeight="1">
       <c r="A91" s="1"/>
       <c r="B91" s="1"/>
       <c r="C91" s="1"/>
@@ -2336,7 +2506,7 @@
       <c r="H91" s="1"/>
       <c r="I91" s="1"/>
     </row>
-    <row r="92" ht="9.75" customHeight="1" spans="1:9">
+    <row r="92" ht="9.75" customHeight="1">
       <c r="A92" s="1"/>
       <c r="B92" s="1"/>
       <c r="C92" s="1"/>
@@ -2347,7 +2517,7 @@
       <c r="H92" s="1"/>
       <c r="I92" s="1"/>
     </row>
-    <row r="93" ht="9.75" customHeight="1" spans="1:9">
+    <row r="93" ht="9.75" customHeight="1">
       <c r="A93" s="1"/>
       <c r="B93" s="1"/>
       <c r="C93" s="1"/>
@@ -2358,7 +2528,7 @@
       <c r="H93" s="1"/>
       <c r="I93" s="1"/>
     </row>
-    <row r="94" ht="9.75" customHeight="1" spans="1:9">
+    <row r="94" ht="9.75" customHeight="1">
       <c r="A94" s="1"/>
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
@@ -2369,7 +2539,7 @@
       <c r="H94" s="1"/>
       <c r="I94" s="1"/>
     </row>
-    <row r="95" ht="9.75" customHeight="1" spans="1:9">
+    <row r="95" ht="9.75" customHeight="1">
       <c r="A95" s="1"/>
       <c r="B95" s="1"/>
       <c r="C95" s="1"/>
@@ -2380,7 +2550,7 @@
       <c r="H95" s="1"/>
       <c r="I95" s="1"/>
     </row>
-    <row r="96" ht="9.75" customHeight="1" spans="1:9">
+    <row r="96" ht="9.75" customHeight="1">
       <c r="A96" s="1"/>
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
@@ -2391,7 +2561,7 @@
       <c r="H96" s="1"/>
       <c r="I96" s="1"/>
     </row>
-    <row r="97" ht="9.75" customHeight="1" spans="1:9">
+    <row r="97" ht="9.75" customHeight="1">
       <c r="A97" s="1"/>
       <c r="B97" s="1"/>
       <c r="C97" s="1"/>
@@ -2402,7 +2572,7 @@
       <c r="H97" s="1"/>
       <c r="I97" s="1"/>
     </row>
-    <row r="98" ht="9.75" customHeight="1" spans="1:9">
+    <row r="98" ht="9.75" customHeight="1">
       <c r="A98" s="1"/>
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
@@ -2413,7 +2583,7 @@
       <c r="H98" s="1"/>
       <c r="I98" s="1"/>
     </row>
-    <row r="99" ht="9.75" customHeight="1" spans="1:9">
+    <row r="99" ht="9.75" customHeight="1">
       <c r="A99" s="1"/>
       <c r="B99" s="1"/>
       <c r="C99" s="1"/>
@@ -2424,7 +2594,7 @@
       <c r="H99" s="1"/>
       <c r="I99" s="1"/>
     </row>
-    <row r="100" ht="9.75" customHeight="1" spans="1:9">
+    <row r="100" ht="9.75" customHeight="1">
       <c r="A100" s="1"/>
       <c r="B100" s="1"/>
       <c r="C100" s="1"/>
@@ -2435,7 +2605,7 @@
       <c r="H100" s="1"/>
       <c r="I100" s="1"/>
     </row>
-    <row r="101" ht="9.75" customHeight="1" spans="1:9">
+    <row r="101" ht="9.75" customHeight="1">
       <c r="A101" s="1"/>
       <c r="B101" s="1"/>
       <c r="C101" s="1"/>
@@ -2446,7 +2616,7 @@
       <c r="H101" s="1"/>
       <c r="I101" s="1"/>
     </row>
-    <row r="102" ht="9.75" customHeight="1" spans="1:9">
+    <row r="102" ht="9.75" customHeight="1">
       <c r="A102" s="1"/>
       <c r="B102" s="1"/>
       <c r="C102" s="1"/>
@@ -2457,7 +2627,7 @@
       <c r="H102" s="1"/>
       <c r="I102" s="1"/>
     </row>
-    <row r="103" ht="9.75" customHeight="1" spans="1:9">
+    <row r="103" ht="9.75" customHeight="1">
       <c r="A103" s="1"/>
       <c r="B103" s="1"/>
       <c r="C103" s="1"/>
@@ -2468,7 +2638,7 @@
       <c r="H103" s="1"/>
       <c r="I103" s="1"/>
     </row>
-    <row r="104" ht="9.75" customHeight="1" spans="1:9">
+    <row r="104" ht="9.75" customHeight="1">
       <c r="A104" s="1"/>
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
@@ -2479,7 +2649,7 @@
       <c r="H104" s="1"/>
       <c r="I104" s="1"/>
     </row>
-    <row r="105" ht="9.75" customHeight="1" spans="1:9">
+    <row r="105" ht="9.75" customHeight="1">
       <c r="A105" s="1"/>
       <c r="B105" s="1"/>
       <c r="C105" s="1"/>
@@ -2490,7 +2660,7 @@
       <c r="H105" s="1"/>
       <c r="I105" s="1"/>
     </row>
-    <row r="106" ht="9.75" customHeight="1" spans="1:9">
+    <row r="106" ht="9.75" customHeight="1">
       <c r="A106" s="1"/>
       <c r="B106" s="1"/>
       <c r="C106" s="1"/>
@@ -2501,7 +2671,7 @@
       <c r="H106" s="1"/>
       <c r="I106" s="1"/>
     </row>
-    <row r="107" ht="9.75" customHeight="1" spans="1:9">
+    <row r="107" ht="9.75" customHeight="1">
       <c r="A107" s="1"/>
       <c r="B107" s="1"/>
       <c r="C107" s="1"/>
@@ -2512,7 +2682,7 @@
       <c r="H107" s="1"/>
       <c r="I107" s="1"/>
     </row>
-    <row r="108" ht="9.75" customHeight="1" spans="1:9">
+    <row r="108" ht="9.75" customHeight="1">
       <c r="A108" s="1"/>
       <c r="B108" s="1"/>
       <c r="C108" s="1"/>
@@ -2523,7 +2693,7 @@
       <c r="H108" s="1"/>
       <c r="I108" s="1"/>
     </row>
-    <row r="109" ht="9.75" customHeight="1" spans="1:9">
+    <row r="109" ht="9.75" customHeight="1">
       <c r="A109" s="1"/>
       <c r="B109" s="1"/>
       <c r="C109" s="1"/>
@@ -2534,7 +2704,7 @@
       <c r="H109" s="1"/>
       <c r="I109" s="1"/>
     </row>
-    <row r="110" ht="9.75" customHeight="1" spans="1:9">
+    <row r="110" ht="9.75" customHeight="1">
       <c r="A110" s="1"/>
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
@@ -2545,7 +2715,7 @@
       <c r="H110" s="1"/>
       <c r="I110" s="1"/>
     </row>
-    <row r="111" ht="9.75" customHeight="1" spans="1:9">
+    <row r="111" ht="9.75" customHeight="1">
       <c r="A111" s="1"/>
       <c r="B111" s="1"/>
       <c r="C111" s="1"/>
@@ -2556,7 +2726,7 @@
       <c r="H111" s="1"/>
       <c r="I111" s="1"/>
     </row>
-    <row r="112" ht="9.75" customHeight="1" spans="1:9">
+    <row r="112" ht="9.75" customHeight="1">
       <c r="A112" s="1"/>
       <c r="B112" s="1"/>
       <c r="C112" s="1"/>
@@ -2567,7 +2737,7 @@
       <c r="H112" s="1"/>
       <c r="I112" s="1"/>
     </row>
-    <row r="113" ht="9.75" customHeight="1" spans="1:9">
+    <row r="113" ht="9.75" customHeight="1">
       <c r="A113" s="1"/>
       <c r="B113" s="1"/>
       <c r="C113" s="1"/>
@@ -2578,7 +2748,7 @@
       <c r="H113" s="1"/>
       <c r="I113" s="1"/>
     </row>
-    <row r="114" ht="9.75" customHeight="1" spans="1:9">
+    <row r="114" ht="9.75" customHeight="1">
       <c r="A114" s="1"/>
       <c r="B114" s="1"/>
       <c r="C114" s="1"/>
@@ -2589,7 +2759,7 @@
       <c r="H114" s="1"/>
       <c r="I114" s="1"/>
     </row>
-    <row r="115" ht="9.75" customHeight="1" spans="1:9">
+    <row r="115" ht="9.75" customHeight="1">
       <c r="A115" s="1"/>
       <c r="B115" s="1"/>
       <c r="C115" s="1"/>
@@ -2600,7 +2770,7 @@
       <c r="H115" s="1"/>
       <c r="I115" s="1"/>
     </row>
-    <row r="116" ht="9.75" customHeight="1" spans="1:9">
+    <row r="116" ht="9.75" customHeight="1">
       <c r="A116" s="1"/>
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
@@ -2611,7 +2781,7 @@
       <c r="H116" s="1"/>
       <c r="I116" s="1"/>
     </row>
-    <row r="117" ht="9.75" customHeight="1" spans="1:9">
+    <row r="117" ht="9.75" customHeight="1">
       <c r="A117" s="1"/>
       <c r="B117" s="1"/>
       <c r="C117" s="1"/>
@@ -2622,7 +2792,7 @@
       <c r="H117" s="1"/>
       <c r="I117" s="1"/>
     </row>
-    <row r="118" ht="9.75" customHeight="1" spans="1:9">
+    <row r="118" ht="9.75" customHeight="1">
       <c r="A118" s="1"/>
       <c r="B118" s="1"/>
       <c r="C118" s="1"/>
@@ -2633,7 +2803,7 @@
       <c r="H118" s="1"/>
       <c r="I118" s="1"/>
     </row>
-    <row r="119" ht="9.75" customHeight="1" spans="1:9">
+    <row r="119" ht="9.75" customHeight="1">
       <c r="A119" s="1"/>
       <c r="B119" s="1"/>
       <c r="C119" s="1"/>
@@ -2644,7 +2814,7 @@
       <c r="H119" s="1"/>
       <c r="I119" s="1"/>
     </row>
-    <row r="120" ht="9.75" customHeight="1" spans="1:9">
+    <row r="120" ht="9.75" customHeight="1">
       <c r="A120" s="1"/>
       <c r="B120" s="1"/>
       <c r="C120" s="1"/>
@@ -2655,7 +2825,7 @@
       <c r="H120" s="1"/>
       <c r="I120" s="1"/>
     </row>
-    <row r="121" ht="9.75" customHeight="1" spans="1:9">
+    <row r="121" ht="9.75" customHeight="1">
       <c r="A121" s="1"/>
       <c r="B121" s="1"/>
       <c r="C121" s="1"/>
@@ -2666,7 +2836,7 @@
       <c r="H121" s="1"/>
       <c r="I121" s="1"/>
     </row>
-    <row r="122" ht="9.75" customHeight="1" spans="1:9">
+    <row r="122" ht="9.75" customHeight="1">
       <c r="A122" s="1"/>
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
@@ -2677,7 +2847,7 @@
       <c r="H122" s="1"/>
       <c r="I122" s="1"/>
     </row>
-    <row r="123" ht="9.75" customHeight="1" spans="1:9">
+    <row r="123" ht="9.75" customHeight="1">
       <c r="A123" s="1"/>
       <c r="B123" s="1"/>
       <c r="C123" s="1"/>
@@ -2688,7 +2858,7 @@
       <c r="H123" s="1"/>
       <c r="I123" s="1"/>
     </row>
-    <row r="124" ht="9.75" customHeight="1" spans="1:9">
+    <row r="124" ht="9.75" customHeight="1">
       <c r="A124" s="1"/>
       <c r="B124" s="1"/>
       <c r="C124" s="1"/>
@@ -2699,7 +2869,7 @@
       <c r="H124" s="1"/>
       <c r="I124" s="1"/>
     </row>
-    <row r="125" ht="9.75" customHeight="1" spans="1:9">
+    <row r="125" ht="9.75" customHeight="1">
       <c r="A125" s="1"/>
       <c r="B125" s="1"/>
       <c r="C125" s="1"/>
@@ -2710,7 +2880,7 @@
       <c r="H125" s="1"/>
       <c r="I125" s="1"/>
     </row>
-    <row r="126" ht="9.75" customHeight="1" spans="1:9">
+    <row r="126" ht="9.75" customHeight="1">
       <c r="A126" s="1"/>
       <c r="B126" s="1"/>
       <c r="C126" s="1"/>
@@ -2721,7 +2891,7 @@
       <c r="H126" s="1"/>
       <c r="I126" s="1"/>
     </row>
-    <row r="127" ht="9.75" customHeight="1" spans="1:9">
+    <row r="127" ht="9.75" customHeight="1">
       <c r="A127" s="1"/>
       <c r="B127" s="1"/>
       <c r="C127" s="1"/>
@@ -2732,7 +2902,7 @@
       <c r="H127" s="1"/>
       <c r="I127" s="1"/>
     </row>
-    <row r="128" ht="9.75" customHeight="1" spans="1:9">
+    <row r="128" ht="9.75" customHeight="1">
       <c r="A128" s="1"/>
       <c r="B128" s="1"/>
       <c r="C128" s="1"/>
@@ -2743,7 +2913,7 @@
       <c r="H128" s="1"/>
       <c r="I128" s="1"/>
     </row>
-    <row r="129" ht="9.75" customHeight="1" spans="1:9">
+    <row r="129" ht="9.75" customHeight="1">
       <c r="A129" s="1"/>
       <c r="B129" s="1"/>
       <c r="C129" s="1"/>
@@ -2754,7 +2924,7 @@
       <c r="H129" s="1"/>
       <c r="I129" s="1"/>
     </row>
-    <row r="130" ht="9.75" customHeight="1" spans="1:9">
+    <row r="130" ht="9.75" customHeight="1">
       <c r="A130" s="1"/>
       <c r="B130" s="1"/>
       <c r="C130" s="1"/>
@@ -2765,7 +2935,7 @@
       <c r="H130" s="1"/>
       <c r="I130" s="1"/>
     </row>
-    <row r="131" ht="9.75" customHeight="1" spans="1:9">
+    <row r="131" ht="9.75" customHeight="1">
       <c r="A131" s="1"/>
       <c r="B131" s="1"/>
       <c r="C131" s="1"/>
@@ -2776,7 +2946,7 @@
       <c r="H131" s="1"/>
       <c r="I131" s="1"/>
     </row>
-    <row r="132" ht="9.75" customHeight="1" spans="1:9">
+    <row r="132" ht="9.75" customHeight="1">
       <c r="A132" s="1"/>
       <c r="B132" s="1"/>
       <c r="C132" s="1"/>
@@ -2787,7 +2957,7 @@
       <c r="H132" s="1"/>
       <c r="I132" s="1"/>
     </row>
-    <row r="133" ht="9.75" customHeight="1" spans="1:9">
+    <row r="133" ht="9.75" customHeight="1">
       <c r="A133" s="1"/>
       <c r="B133" s="1"/>
       <c r="C133" s="1"/>
@@ -2798,7 +2968,7 @@
       <c r="H133" s="1"/>
       <c r="I133" s="1"/>
     </row>
-    <row r="134" ht="9.75" customHeight="1" spans="1:9">
+    <row r="134" ht="9.75" customHeight="1">
       <c r="A134" s="1"/>
       <c r="B134" s="1"/>
       <c r="C134" s="1"/>
@@ -2809,7 +2979,7 @@
       <c r="H134" s="1"/>
       <c r="I134" s="1"/>
     </row>
-    <row r="135" ht="9.75" customHeight="1" spans="1:9">
+    <row r="135" ht="9.75" customHeight="1">
       <c r="A135" s="1"/>
       <c r="B135" s="1"/>
       <c r="C135" s="1"/>
@@ -2820,7 +2990,7 @@
       <c r="H135" s="1"/>
       <c r="I135" s="1"/>
     </row>
-    <row r="136" ht="9.75" customHeight="1" spans="1:9">
+    <row r="136" ht="9.75" customHeight="1">
       <c r="A136" s="1"/>
       <c r="B136" s="1"/>
       <c r="C136" s="1"/>
@@ -2831,7 +3001,7 @@
       <c r="H136" s="1"/>
       <c r="I136" s="1"/>
     </row>
-    <row r="137" ht="9.75" customHeight="1" spans="1:9">
+    <row r="137" ht="9.75" customHeight="1">
       <c r="A137" s="1"/>
       <c r="B137" s="1"/>
       <c r="C137" s="1"/>
@@ -2842,7 +3012,7 @@
       <c r="H137" s="1"/>
       <c r="I137" s="1"/>
     </row>
-    <row r="138" ht="9.75" customHeight="1" spans="1:9">
+    <row r="138" ht="9.75" customHeight="1">
       <c r="A138" s="1"/>
       <c r="B138" s="1"/>
       <c r="C138" s="1"/>
@@ -2853,7 +3023,7 @@
       <c r="H138" s="1"/>
       <c r="I138" s="1"/>
     </row>
-    <row r="139" ht="9.75" customHeight="1" spans="1:9">
+    <row r="139" ht="9.75" customHeight="1">
       <c r="A139" s="1"/>
       <c r="B139" s="1"/>
       <c r="C139" s="1"/>
@@ -2864,7 +3034,7 @@
       <c r="H139" s="1"/>
       <c r="I139" s="1"/>
     </row>
-    <row r="140" ht="9.75" customHeight="1" spans="1:9">
+    <row r="140" ht="9.75" customHeight="1">
       <c r="A140" s="1"/>
       <c r="B140" s="1"/>
       <c r="C140" s="1"/>
@@ -2875,7 +3045,7 @@
       <c r="H140" s="1"/>
       <c r="I140" s="1"/>
     </row>
-    <row r="141" ht="9.75" customHeight="1" spans="1:9">
+    <row r="141" ht="9.75" customHeight="1">
       <c r="A141" s="1"/>
       <c r="B141" s="1"/>
       <c r="C141" s="1"/>
@@ -2886,7 +3056,7 @@
       <c r="H141" s="1"/>
       <c r="I141" s="1"/>
     </row>
-    <row r="142" ht="9.75" customHeight="1" spans="1:9">
+    <row r="142" ht="9.75" customHeight="1">
       <c r="A142" s="1"/>
       <c r="B142" s="1"/>
       <c r="C142" s="1"/>
@@ -2897,7 +3067,7 @@
       <c r="H142" s="1"/>
       <c r="I142" s="1"/>
     </row>
-    <row r="143" ht="9.75" customHeight="1" spans="1:9">
+    <row r="143" ht="9.75" customHeight="1">
       <c r="A143" s="1"/>
       <c r="B143" s="1"/>
       <c r="C143" s="1"/>
@@ -2908,7 +3078,7 @@
       <c r="H143" s="1"/>
       <c r="I143" s="1"/>
     </row>
-    <row r="144" ht="9.75" customHeight="1" spans="1:9">
+    <row r="144" ht="9.75" customHeight="1">
       <c r="A144" s="1"/>
       <c r="B144" s="1"/>
       <c r="C144" s="1"/>
@@ -2919,7 +3089,7 @@
       <c r="H144" s="1"/>
       <c r="I144" s="1"/>
     </row>
-    <row r="145" ht="9.75" customHeight="1" spans="1:9">
+    <row r="145" ht="9.75" customHeight="1">
       <c r="A145" s="1"/>
       <c r="B145" s="1"/>
       <c r="C145" s="1"/>
@@ -2930,7 +3100,7 @@
       <c r="H145" s="1"/>
       <c r="I145" s="1"/>
     </row>
-    <row r="146" ht="9.75" customHeight="1" spans="1:9">
+    <row r="146" ht="9.75" customHeight="1">
       <c r="A146" s="1"/>
       <c r="B146" s="1"/>
       <c r="C146" s="1"/>
@@ -2941,7 +3111,7 @@
       <c r="H146" s="1"/>
       <c r="I146" s="1"/>
     </row>
-    <row r="147" ht="9.75" customHeight="1" spans="1:9">
+    <row r="147" ht="9.75" customHeight="1">
       <c r="A147" s="1"/>
       <c r="B147" s="1"/>
       <c r="C147" s="1"/>
@@ -2952,7 +3122,7 @@
       <c r="H147" s="1"/>
       <c r="I147" s="1"/>
     </row>
-    <row r="148" ht="9.75" customHeight="1" spans="1:9">
+    <row r="148" ht="9.75" customHeight="1">
       <c r="A148" s="1"/>
       <c r="B148" s="1"/>
       <c r="C148" s="1"/>
@@ -2963,7 +3133,7 @@
       <c r="H148" s="1"/>
       <c r="I148" s="1"/>
     </row>
-    <row r="149" ht="9.75" customHeight="1" spans="1:9">
+    <row r="149" ht="9.75" customHeight="1">
       <c r="A149" s="1"/>
       <c r="B149" s="1"/>
       <c r="C149" s="1"/>
@@ -2974,7 +3144,7 @@
       <c r="H149" s="1"/>
       <c r="I149" s="1"/>
     </row>
-    <row r="150" ht="9.75" customHeight="1" spans="1:9">
+    <row r="150" ht="9.75" customHeight="1">
       <c r="A150" s="1"/>
       <c r="B150" s="1"/>
       <c r="C150" s="1"/>
@@ -2985,7 +3155,7 @@
       <c r="H150" s="1"/>
       <c r="I150" s="1"/>
     </row>
-    <row r="151" ht="9.75" customHeight="1" spans="1:9">
+    <row r="151" ht="9.75" customHeight="1">
       <c r="A151" s="1"/>
       <c r="B151" s="1"/>
       <c r="C151" s="1"/>
@@ -2996,7 +3166,7 @@
       <c r="H151" s="1"/>
       <c r="I151" s="1"/>
     </row>
-    <row r="152" ht="9.75" customHeight="1" spans="1:9">
+    <row r="152" ht="9.75" customHeight="1">
       <c r="A152" s="1"/>
       <c r="B152" s="1"/>
       <c r="C152" s="1"/>
@@ -3007,7 +3177,7 @@
       <c r="H152" s="1"/>
       <c r="I152" s="1"/>
     </row>
-    <row r="153" ht="9.75" customHeight="1" spans="1:9">
+    <row r="153" ht="9.75" customHeight="1">
       <c r="A153" s="1"/>
       <c r="B153" s="1"/>
       <c r="C153" s="1"/>
@@ -3018,7 +3188,7 @@
       <c r="H153" s="1"/>
       <c r="I153" s="1"/>
     </row>
-    <row r="154" ht="9.75" customHeight="1" spans="1:9">
+    <row r="154" ht="9.75" customHeight="1">
       <c r="A154" s="1"/>
       <c r="B154" s="1"/>
       <c r="C154" s="1"/>
@@ -3029,7 +3199,7 @@
       <c r="H154" s="1"/>
       <c r="I154" s="1"/>
     </row>
-    <row r="155" ht="9.75" customHeight="1" spans="1:9">
+    <row r="155" ht="9.75" customHeight="1">
       <c r="A155" s="1"/>
       <c r="B155" s="1"/>
       <c r="C155" s="1"/>
@@ -3040,7 +3210,7 @@
       <c r="H155" s="1"/>
       <c r="I155" s="1"/>
     </row>
-    <row r="156" ht="9.75" customHeight="1" spans="1:9">
+    <row r="156" ht="9.75" customHeight="1">
       <c r="A156" s="1"/>
       <c r="B156" s="1"/>
       <c r="C156" s="1"/>
@@ -3051,7 +3221,7 @@
       <c r="H156" s="1"/>
       <c r="I156" s="1"/>
     </row>
-    <row r="157" ht="9.75" customHeight="1" spans="1:9">
+    <row r="157" ht="9.75" customHeight="1">
       <c r="A157" s="1"/>
       <c r="B157" s="1"/>
       <c r="C157" s="1"/>
@@ -3062,7 +3232,7 @@
       <c r="H157" s="1"/>
       <c r="I157" s="1"/>
     </row>
-    <row r="158" ht="9.75" customHeight="1" spans="1:9">
+    <row r="158" ht="9.75" customHeight="1">
       <c r="A158" s="1"/>
       <c r="B158" s="1"/>
       <c r="C158" s="1"/>
@@ -3073,7 +3243,7 @@
       <c r="H158" s="1"/>
       <c r="I158" s="1"/>
     </row>
-    <row r="159" ht="9.75" customHeight="1" spans="1:9">
+    <row r="159" ht="9.75" customHeight="1">
       <c r="A159" s="1"/>
       <c r="B159" s="1"/>
       <c r="C159" s="1"/>
@@ -3084,7 +3254,7 @@
       <c r="H159" s="1"/>
       <c r="I159" s="1"/>
     </row>
-    <row r="160" ht="9.75" customHeight="1" spans="1:9">
+    <row r="160" ht="9.75" customHeight="1">
       <c r="A160" s="1"/>
       <c r="B160" s="1"/>
       <c r="C160" s="1"/>
@@ -3095,7 +3265,7 @@
       <c r="H160" s="1"/>
       <c r="I160" s="1"/>
     </row>
-    <row r="161" ht="9.75" customHeight="1" spans="1:9">
+    <row r="161" ht="9.75" customHeight="1">
       <c r="A161" s="1"/>
       <c r="B161" s="1"/>
       <c r="C161" s="1"/>
@@ -3106,7 +3276,7 @@
       <c r="H161" s="1"/>
       <c r="I161" s="1"/>
     </row>
-    <row r="162" ht="9.75" customHeight="1" spans="1:9">
+    <row r="162" ht="9.75" customHeight="1">
       <c r="A162" s="1"/>
       <c r="B162" s="1"/>
       <c r="C162" s="1"/>
@@ -3117,7 +3287,7 @@
       <c r="H162" s="1"/>
       <c r="I162" s="1"/>
     </row>
-    <row r="163" ht="9.75" customHeight="1" spans="1:9">
+    <row r="163" ht="9.75" customHeight="1">
       <c r="A163" s="1"/>
       <c r="B163" s="1"/>
       <c r="C163" s="1"/>
@@ -3128,7 +3298,7 @@
       <c r="H163" s="1"/>
       <c r="I163" s="1"/>
     </row>
-    <row r="164" ht="9.75" customHeight="1" spans="1:9">
+    <row r="164" ht="9.75" customHeight="1">
       <c r="A164" s="1"/>
       <c r="B164" s="1"/>
       <c r="C164" s="1"/>
@@ -3139,7 +3309,7 @@
       <c r="H164" s="1"/>
       <c r="I164" s="1"/>
     </row>
-    <row r="165" ht="9.75" customHeight="1" spans="1:9">
+    <row r="165" ht="9.75" customHeight="1">
       <c r="A165" s="1"/>
       <c r="B165" s="1"/>
       <c r="C165" s="1"/>
@@ -3150,7 +3320,7 @@
       <c r="H165" s="1"/>
       <c r="I165" s="1"/>
     </row>
-    <row r="166" ht="9.75" customHeight="1" spans="1:9">
+    <row r="166" ht="9.75" customHeight="1">
       <c r="A166" s="1"/>
       <c r="B166" s="1"/>
       <c r="C166" s="1"/>
@@ -3161,7 +3331,7 @@
       <c r="H166" s="1"/>
       <c r="I166" s="1"/>
     </row>
-    <row r="167" ht="9.75" customHeight="1" spans="1:9">
+    <row r="167" ht="9.75" customHeight="1">
       <c r="A167" s="1"/>
       <c r="B167" s="1"/>
       <c r="C167" s="1"/>
@@ -3172,7 +3342,7 @@
       <c r="H167" s="1"/>
       <c r="I167" s="1"/>
     </row>
-    <row r="168" ht="9.75" customHeight="1" spans="1:9">
+    <row r="168" ht="9.75" customHeight="1">
       <c r="A168" s="1"/>
       <c r="B168" s="1"/>
       <c r="C168" s="1"/>
@@ -3183,7 +3353,7 @@
       <c r="H168" s="1"/>
       <c r="I168" s="1"/>
     </row>
-    <row r="169" ht="9.75" customHeight="1" spans="1:9">
+    <row r="169" ht="9.75" customHeight="1">
       <c r="A169" s="1"/>
       <c r="B169" s="1"/>
       <c r="C169" s="1"/>
@@ -3194,7 +3364,7 @@
       <c r="H169" s="1"/>
       <c r="I169" s="1"/>
     </row>
-    <row r="170" ht="9.75" customHeight="1" spans="1:9">
+    <row r="170" ht="9.75" customHeight="1">
       <c r="A170" s="1"/>
       <c r="B170" s="1"/>
       <c r="C170" s="1"/>
@@ -3205,7 +3375,7 @@
       <c r="H170" s="1"/>
       <c r="I170" s="1"/>
     </row>
-    <row r="171" ht="9.75" customHeight="1" spans="1:9">
+    <row r="171" ht="9.75" customHeight="1">
       <c r="A171" s="1"/>
       <c r="B171" s="1"/>
       <c r="C171" s="1"/>
@@ -3216,7 +3386,7 @@
       <c r="H171" s="1"/>
       <c r="I171" s="1"/>
     </row>
-    <row r="172" ht="9.75" customHeight="1" spans="1:9">
+    <row r="172" ht="9.75" customHeight="1">
       <c r="A172" s="1"/>
       <c r="B172" s="1"/>
       <c r="C172" s="1"/>
@@ -3227,7 +3397,7 @@
       <c r="H172" s="1"/>
       <c r="I172" s="1"/>
     </row>
-    <row r="173" ht="9.75" customHeight="1" spans="1:9">
+    <row r="173" ht="9.75" customHeight="1">
       <c r="A173" s="1"/>
       <c r="B173" s="1"/>
       <c r="C173" s="1"/>
@@ -3238,7 +3408,7 @@
       <c r="H173" s="1"/>
       <c r="I173" s="1"/>
     </row>
-    <row r="174" ht="9.75" customHeight="1" spans="1:9">
+    <row r="174" ht="9.75" customHeight="1">
       <c r="A174" s="1"/>
       <c r="B174" s="1"/>
       <c r="C174" s="1"/>
@@ -3249,7 +3419,7 @@
       <c r="H174" s="1"/>
       <c r="I174" s="1"/>
     </row>
-    <row r="175" ht="9.75" customHeight="1" spans="1:9">
+    <row r="175" ht="9.75" customHeight="1">
       <c r="A175" s="1"/>
       <c r="B175" s="1"/>
       <c r="C175" s="1"/>
@@ -3260,7 +3430,7 @@
       <c r="H175" s="1"/>
       <c r="I175" s="1"/>
     </row>
-    <row r="176" ht="9.75" customHeight="1" spans="1:9">
+    <row r="176" ht="9.75" customHeight="1">
       <c r="A176" s="1"/>
       <c r="B176" s="1"/>
       <c r="C176" s="1"/>
@@ -3271,7 +3441,7 @@
       <c r="H176" s="1"/>
       <c r="I176" s="1"/>
     </row>
-    <row r="177" ht="9.75" customHeight="1" spans="1:9">
+    <row r="177" ht="9.75" customHeight="1">
       <c r="A177" s="1"/>
       <c r="B177" s="1"/>
       <c r="C177" s="1"/>
@@ -3282,7 +3452,7 @@
       <c r="H177" s="1"/>
       <c r="I177" s="1"/>
     </row>
-    <row r="178" ht="9.75" customHeight="1" spans="1:9">
+    <row r="178" ht="9.75" customHeight="1">
       <c r="A178" s="1"/>
       <c r="B178" s="1"/>
       <c r="C178" s="1"/>
@@ -3293,7 +3463,7 @@
       <c r="H178" s="1"/>
       <c r="I178" s="1"/>
     </row>
-    <row r="179" ht="9.75" customHeight="1" spans="1:9">
+    <row r="179" ht="9.75" customHeight="1">
       <c r="A179" s="1"/>
       <c r="B179" s="1"/>
       <c r="C179" s="1"/>
@@ -3304,7 +3474,7 @@
       <c r="H179" s="1"/>
       <c r="I179" s="1"/>
     </row>
-    <row r="180" ht="9.75" customHeight="1" spans="1:9">
+    <row r="180" ht="9.75" customHeight="1">
       <c r="A180" s="1"/>
       <c r="B180" s="1"/>
       <c r="C180" s="1"/>
@@ -3315,7 +3485,7 @@
       <c r="H180" s="1"/>
       <c r="I180" s="1"/>
     </row>
-    <row r="181" ht="9.75" customHeight="1" spans="1:9">
+    <row r="181" ht="9.75" customHeight="1">
       <c r="A181" s="1"/>
       <c r="B181" s="1"/>
       <c r="C181" s="1"/>
@@ -3326,7 +3496,7 @@
       <c r="H181" s="1"/>
       <c r="I181" s="1"/>
     </row>
-    <row r="182" ht="9.75" customHeight="1" spans="1:9">
+    <row r="182" ht="9.75" customHeight="1">
       <c r="A182" s="1"/>
       <c r="B182" s="1"/>
       <c r="C182" s="1"/>
@@ -3337,7 +3507,7 @@
       <c r="H182" s="1"/>
       <c r="I182" s="1"/>
     </row>
-    <row r="183" ht="9.75" customHeight="1" spans="1:9">
+    <row r="183" ht="9.75" customHeight="1">
       <c r="A183" s="1"/>
       <c r="B183" s="1"/>
       <c r="C183" s="1"/>
@@ -3348,7 +3518,7 @@
       <c r="H183" s="1"/>
       <c r="I183" s="1"/>
     </row>
-    <row r="184" ht="9.75" customHeight="1" spans="1:9">
+    <row r="184" ht="9.75" customHeight="1">
       <c r="A184" s="1"/>
       <c r="B184" s="1"/>
       <c r="C184" s="1"/>
@@ -3359,7 +3529,7 @@
       <c r="H184" s="1"/>
       <c r="I184" s="1"/>
     </row>
-    <row r="185" ht="9.75" customHeight="1" spans="1:9">
+    <row r="185" ht="9.75" customHeight="1">
       <c r="A185" s="1"/>
       <c r="B185" s="1"/>
       <c r="C185" s="1"/>
@@ -3370,7 +3540,7 @@
       <c r="H185" s="1"/>
       <c r="I185" s="1"/>
     </row>
-    <row r="186" ht="9.75" customHeight="1" spans="1:9">
+    <row r="186" ht="9.75" customHeight="1">
       <c r="A186" s="1"/>
       <c r="B186" s="1"/>
       <c r="C186" s="1"/>
@@ -3381,7 +3551,7 @@
       <c r="H186" s="1"/>
       <c r="I186" s="1"/>
     </row>
-    <row r="187" ht="9.75" customHeight="1" spans="1:9">
+    <row r="187" ht="9.75" customHeight="1">
       <c r="A187" s="1"/>
       <c r="B187" s="1"/>
       <c r="C187" s="1"/>
@@ -3392,7 +3562,7 @@
       <c r="H187" s="1"/>
       <c r="I187" s="1"/>
     </row>
-    <row r="188" ht="9.75" customHeight="1" spans="1:9">
+    <row r="188" ht="9.75" customHeight="1">
       <c r="A188" s="1"/>
       <c r="B188" s="1"/>
       <c r="C188" s="1"/>
@@ -3403,7 +3573,7 @@
       <c r="H188" s="1"/>
       <c r="I188" s="1"/>
     </row>
-    <row r="189" ht="9.75" customHeight="1" spans="1:9">
+    <row r="189" ht="9.75" customHeight="1">
       <c r="A189" s="1"/>
       <c r="B189" s="1"/>
       <c r="C189" s="1"/>
@@ -3414,7 +3584,7 @@
       <c r="H189" s="1"/>
       <c r="I189" s="1"/>
     </row>
-    <row r="190" ht="9.75" customHeight="1" spans="1:9">
+    <row r="190" ht="9.75" customHeight="1">
       <c r="A190" s="1"/>
       <c r="B190" s="1"/>
       <c r="C190" s="1"/>
@@ -3425,7 +3595,7 @@
       <c r="H190" s="1"/>
       <c r="I190" s="1"/>
     </row>
-    <row r="191" ht="9.75" customHeight="1" spans="1:9">
+    <row r="191" ht="9.75" customHeight="1">
       <c r="A191" s="1"/>
       <c r="B191" s="1"/>
       <c r="C191" s="1"/>
@@ -3436,7 +3606,7 @@
       <c r="H191" s="1"/>
       <c r="I191" s="1"/>
     </row>
-    <row r="192" ht="9.75" customHeight="1" spans="1:9">
+    <row r="192" ht="9.75" customHeight="1">
       <c r="A192" s="1"/>
       <c r="B192" s="1"/>
       <c r="C192" s="1"/>
@@ -3447,7 +3617,7 @@
       <c r="H192" s="1"/>
       <c r="I192" s="1"/>
     </row>
-    <row r="193" ht="9.75" customHeight="1" spans="1:9">
+    <row r="193" ht="9.75" customHeight="1">
       <c r="A193" s="1"/>
       <c r="B193" s="1"/>
       <c r="C193" s="1"/>
@@ -3458,7 +3628,7 @@
       <c r="H193" s="1"/>
       <c r="I193" s="1"/>
     </row>
-    <row r="194" ht="9.75" customHeight="1" spans="1:9">
+    <row r="194" ht="9.75" customHeight="1">
       <c r="A194" s="1"/>
       <c r="B194" s="1"/>
       <c r="C194" s="1"/>
@@ -3469,7 +3639,7 @@
       <c r="H194" s="1"/>
       <c r="I194" s="1"/>
     </row>
-    <row r="195" ht="9.75" customHeight="1" spans="1:9">
+    <row r="195" ht="9.75" customHeight="1">
       <c r="A195" s="1"/>
       <c r="B195" s="1"/>
       <c r="C195" s="1"/>
@@ -3480,7 +3650,7 @@
       <c r="H195" s="1"/>
       <c r="I195" s="1"/>
     </row>
-    <row r="196" ht="9.75" customHeight="1" spans="1:9">
+    <row r="196" ht="9.75" customHeight="1">
       <c r="A196" s="1"/>
       <c r="B196" s="1"/>
       <c r="C196" s="1"/>
@@ -3491,7 +3661,7 @@
       <c r="H196" s="1"/>
       <c r="I196" s="1"/>
     </row>
-    <row r="197" ht="9.75" customHeight="1" spans="1:9">
+    <row r="197" ht="9.75" customHeight="1">
       <c r="A197" s="1"/>
       <c r="B197" s="1"/>
       <c r="C197" s="1"/>
@@ -3502,7 +3672,7 @@
       <c r="H197" s="1"/>
       <c r="I197" s="1"/>
     </row>
-    <row r="198" ht="9.75" customHeight="1" spans="1:9">
+    <row r="198" ht="9.75" customHeight="1">
       <c r="A198" s="1"/>
       <c r="B198" s="1"/>
       <c r="C198" s="1"/>
@@ -3513,7 +3683,7 @@
       <c r="H198" s="1"/>
       <c r="I198" s="1"/>
     </row>
-    <row r="199" ht="9.75" customHeight="1" spans="1:9">
+    <row r="199" ht="9.75" customHeight="1">
       <c r="A199" s="1"/>
       <c r="B199" s="1"/>
       <c r="C199" s="1"/>
@@ -3524,7 +3694,7 @@
       <c r="H199" s="1"/>
       <c r="I199" s="1"/>
     </row>
-    <row r="200" ht="9.75" customHeight="1" spans="1:9">
+    <row r="200" ht="9.75" customHeight="1">
       <c r="A200" s="1"/>
       <c r="B200" s="1"/>
       <c r="C200" s="1"/>
@@ -3535,7 +3705,7 @@
       <c r="H200" s="1"/>
       <c r="I200" s="1"/>
     </row>
-    <row r="201" ht="9.75" customHeight="1" spans="1:9">
+    <row r="201" ht="9.75" customHeight="1">
       <c r="A201" s="1"/>
       <c r="B201" s="1"/>
       <c r="C201" s="1"/>
@@ -3546,7 +3716,7 @@
       <c r="H201" s="1"/>
       <c r="I201" s="1"/>
     </row>
-    <row r="202" ht="9.75" customHeight="1" spans="1:9">
+    <row r="202" ht="9.75" customHeight="1">
       <c r="A202" s="1"/>
       <c r="B202" s="1"/>
       <c r="C202" s="1"/>
@@ -3557,7 +3727,7 @@
       <c r="H202" s="1"/>
       <c r="I202" s="1"/>
     </row>
-    <row r="203" ht="9.75" customHeight="1" spans="1:9">
+    <row r="203" ht="9.75" customHeight="1">
       <c r="A203" s="1"/>
       <c r="B203" s="1"/>
       <c r="C203" s="1"/>
@@ -3568,7 +3738,7 @@
       <c r="H203" s="1"/>
       <c r="I203" s="1"/>
     </row>
-    <row r="204" ht="9.75" customHeight="1" spans="1:9">
+    <row r="204" ht="9.75" customHeight="1">
       <c r="A204" s="1"/>
       <c r="B204" s="1"/>
       <c r="C204" s="1"/>
@@ -3579,7 +3749,7 @@
       <c r="H204" s="1"/>
       <c r="I204" s="1"/>
     </row>
-    <row r="205" ht="9.75" customHeight="1" spans="1:9">
+    <row r="205" ht="9.75" customHeight="1">
       <c r="A205" s="1"/>
       <c r="B205" s="1"/>
       <c r="C205" s="1"/>
@@ -3590,7 +3760,7 @@
       <c r="H205" s="1"/>
       <c r="I205" s="1"/>
     </row>
-    <row r="206" ht="9.75" customHeight="1" spans="1:9">
+    <row r="206" ht="9.75" customHeight="1">
       <c r="A206" s="1"/>
       <c r="B206" s="1"/>
       <c r="C206" s="1"/>
@@ -3601,7 +3771,7 @@
       <c r="H206" s="1"/>
       <c r="I206" s="1"/>
     </row>
-    <row r="207" ht="9.75" customHeight="1" spans="1:9">
+    <row r="207" ht="9.75" customHeight="1">
       <c r="A207" s="1"/>
       <c r="B207" s="1"/>
       <c r="C207" s="1"/>
@@ -3612,7 +3782,7 @@
       <c r="H207" s="1"/>
       <c r="I207" s="1"/>
     </row>
-    <row r="208" ht="9.75" customHeight="1" spans="1:9">
+    <row r="208" ht="9.75" customHeight="1">
       <c r="A208" s="1"/>
       <c r="B208" s="1"/>
       <c r="C208" s="1"/>
@@ -3623,7 +3793,7 @@
       <c r="H208" s="1"/>
       <c r="I208" s="1"/>
     </row>
-    <row r="209" ht="9.75" customHeight="1" spans="1:9">
+    <row r="209" ht="9.75" customHeight="1">
       <c r="A209" s="1"/>
       <c r="B209" s="1"/>
       <c r="C209" s="1"/>
@@ -3634,7 +3804,7 @@
       <c r="H209" s="1"/>
       <c r="I209" s="1"/>
     </row>
-    <row r="210" ht="9.75" customHeight="1" spans="1:9">
+    <row r="210" ht="9.75" customHeight="1">
       <c r="A210" s="1"/>
       <c r="B210" s="1"/>
       <c r="C210" s="1"/>
@@ -3645,7 +3815,7 @@
       <c r="H210" s="1"/>
       <c r="I210" s="1"/>
     </row>
-    <row r="211" ht="9.75" customHeight="1" spans="1:9">
+    <row r="211" ht="9.75" customHeight="1">
       <c r="A211" s="1"/>
       <c r="B211" s="1"/>
       <c r="C211" s="1"/>
@@ -3656,7 +3826,7 @@
       <c r="H211" s="1"/>
       <c r="I211" s="1"/>
     </row>
-    <row r="212" ht="9.75" customHeight="1" spans="1:9">
+    <row r="212" ht="9.75" customHeight="1">
       <c r="A212" s="1"/>
       <c r="B212" s="1"/>
       <c r="C212" s="1"/>
@@ -3667,7 +3837,7 @@
       <c r="H212" s="1"/>
       <c r="I212" s="1"/>
     </row>
-    <row r="213" ht="9.75" customHeight="1" spans="1:9">
+    <row r="213" ht="9.75" customHeight="1">
       <c r="A213" s="1"/>
       <c r="B213" s="1"/>
       <c r="C213" s="1"/>
@@ -3678,7 +3848,7 @@
       <c r="H213" s="1"/>
       <c r="I213" s="1"/>
     </row>
-    <row r="214" ht="9.75" customHeight="1" spans="1:9">
+    <row r="214" ht="9.75" customHeight="1">
       <c r="A214" s="1"/>
       <c r="B214" s="1"/>
       <c r="C214" s="1"/>
@@ -3689,7 +3859,7 @@
       <c r="H214" s="1"/>
       <c r="I214" s="1"/>
     </row>
-    <row r="215" ht="9.75" customHeight="1" spans="1:9">
+    <row r="215" ht="9.75" customHeight="1">
       <c r="A215" s="1"/>
       <c r="B215" s="1"/>
       <c r="C215" s="1"/>
@@ -3700,7 +3870,7 @@
       <c r="H215" s="1"/>
       <c r="I215" s="1"/>
     </row>
-    <row r="216" ht="9.75" customHeight="1" spans="1:9">
+    <row r="216" ht="9.75" customHeight="1">
       <c r="A216" s="1"/>
       <c r="B216" s="1"/>
       <c r="C216" s="1"/>
@@ -3711,7 +3881,7 @@
       <c r="H216" s="1"/>
       <c r="I216" s="1"/>
     </row>
-    <row r="217" ht="9.75" customHeight="1" spans="1:9">
+    <row r="217" ht="9.75" customHeight="1">
       <c r="A217" s="1"/>
       <c r="B217" s="1"/>
       <c r="C217" s="1"/>
@@ -3722,7 +3892,7 @@
       <c r="H217" s="1"/>
       <c r="I217" s="1"/>
     </row>
-    <row r="218" ht="9.75" customHeight="1" spans="1:9">
+    <row r="218" ht="9.75" customHeight="1">
       <c r="A218" s="1"/>
       <c r="B218" s="1"/>
       <c r="C218" s="1"/>
@@ -3733,7 +3903,7 @@
       <c r="H218" s="1"/>
       <c r="I218" s="1"/>
     </row>
-    <row r="219" ht="9.75" customHeight="1" spans="1:9">
+    <row r="219" ht="9.75" customHeight="1">
       <c r="A219" s="1"/>
       <c r="B219" s="1"/>
       <c r="C219" s="1"/>
@@ -3744,7 +3914,7 @@
       <c r="H219" s="1"/>
       <c r="I219" s="1"/>
     </row>
-    <row r="220" ht="9.75" customHeight="1" spans="1:9">
+    <row r="220" ht="9.75" customHeight="1">
       <c r="A220" s="1"/>
       <c r="B220" s="1"/>
       <c r="C220" s="1"/>
@@ -3755,7 +3925,7 @@
       <c r="H220" s="1"/>
       <c r="I220" s="1"/>
     </row>
-    <row r="221" ht="9.75" customHeight="1" spans="1:9">
+    <row r="221" ht="9.75" customHeight="1">
       <c r="A221" s="1"/>
       <c r="B221" s="1"/>
       <c r="C221" s="1"/>
@@ -3766,7 +3936,7 @@
       <c r="H221" s="1"/>
       <c r="I221" s="1"/>
     </row>
-    <row r="222" ht="9.75" customHeight="1" spans="1:9">
+    <row r="222" ht="9.75" customHeight="1">
       <c r="A222" s="1"/>
       <c r="B222" s="1"/>
       <c r="C222" s="1"/>
@@ -3777,7 +3947,7 @@
       <c r="H222" s="1"/>
       <c r="I222" s="1"/>
     </row>
-    <row r="223" ht="9.75" customHeight="1" spans="1:9">
+    <row r="223" ht="9.75" customHeight="1">
       <c r="A223" s="1"/>
       <c r="B223" s="1"/>
       <c r="C223" s="1"/>
@@ -3788,7 +3958,7 @@
       <c r="H223" s="1"/>
       <c r="I223" s="1"/>
     </row>
-    <row r="224" ht="9.75" customHeight="1" spans="1:9">
+    <row r="224" ht="9.75" customHeight="1">
       <c r="A224" s="1"/>
       <c r="B224" s="1"/>
       <c r="C224" s="1"/>
@@ -3799,7 +3969,7 @@
       <c r="H224" s="1"/>
       <c r="I224" s="1"/>
     </row>
-    <row r="225" ht="9.75" customHeight="1" spans="1:9">
+    <row r="225" ht="9.75" customHeight="1">
       <c r="A225" s="1"/>
       <c r="B225" s="1"/>
       <c r="C225" s="1"/>
@@ -3810,7 +3980,7 @@
       <c r="H225" s="1"/>
       <c r="I225" s="1"/>
     </row>
-    <row r="226" ht="9.75" customHeight="1" spans="1:9">
+    <row r="226" ht="9.75" customHeight="1">
       <c r="A226" s="1"/>
       <c r="B226" s="1"/>
       <c r="C226" s="1"/>
@@ -3821,7 +3991,7 @@
       <c r="H226" s="1"/>
       <c r="I226" s="1"/>
     </row>
-    <row r="227" ht="9.75" customHeight="1" spans="1:9">
+    <row r="227" ht="9.75" customHeight="1">
       <c r="A227" s="1"/>
       <c r="B227" s="1"/>
       <c r="C227" s="1"/>
@@ -3832,7 +4002,7 @@
       <c r="H227" s="1"/>
       <c r="I227" s="1"/>
     </row>
-    <row r="228" ht="9.75" customHeight="1" spans="1:9">
+    <row r="228" ht="9.75" customHeight="1">
       <c r="A228" s="1"/>
       <c r="B228" s="1"/>
       <c r="C228" s="1"/>
@@ -3843,7 +4013,7 @@
       <c r="H228" s="1"/>
       <c r="I228" s="1"/>
     </row>
-    <row r="229" ht="9.75" customHeight="1" spans="1:9">
+    <row r="229" ht="9.75" customHeight="1">
       <c r="A229" s="1"/>
       <c r="B229" s="1"/>
       <c r="C229" s="1"/>
@@ -3854,7 +4024,7 @@
       <c r="H229" s="1"/>
       <c r="I229" s="1"/>
     </row>
-    <row r="230" ht="9.75" customHeight="1" spans="1:9">
+    <row r="230" ht="9.75" customHeight="1">
       <c r="A230" s="1"/>
       <c r="B230" s="1"/>
       <c r="C230" s="1"/>
@@ -3865,7 +4035,7 @@
       <c r="H230" s="1"/>
       <c r="I230" s="1"/>
     </row>
-    <row r="231" ht="9.75" customHeight="1" spans="1:9">
+    <row r="231" ht="9.75" customHeight="1">
       <c r="A231" s="1"/>
       <c r="B231" s="1"/>
       <c r="C231" s="1"/>
@@ -3876,7 +4046,7 @@
       <c r="H231" s="1"/>
       <c r="I231" s="1"/>
     </row>
-    <row r="232" ht="9.75" customHeight="1" spans="1:9">
+    <row r="232" ht="9.75" customHeight="1">
       <c r="A232" s="1"/>
       <c r="B232" s="1"/>
       <c r="C232" s="1"/>
@@ -3887,7 +4057,7 @@
       <c r="H232" s="1"/>
       <c r="I232" s="1"/>
     </row>
-    <row r="233" ht="9.75" customHeight="1" spans="1:9">
+    <row r="233" ht="9.75" customHeight="1">
       <c r="A233" s="1"/>
       <c r="B233" s="1"/>
       <c r="C233" s="1"/>
@@ -3898,7 +4068,7 @@
       <c r="H233" s="1"/>
       <c r="I233" s="1"/>
     </row>
-    <row r="234" ht="9.75" customHeight="1" spans="1:9">
+    <row r="234" ht="9.75" customHeight="1">
       <c r="A234" s="1"/>
       <c r="B234" s="1"/>
       <c r="C234" s="1"/>
@@ -3909,7 +4079,7 @@
       <c r="H234" s="1"/>
       <c r="I234" s="1"/>
     </row>
-    <row r="235" ht="9.75" customHeight="1" spans="1:9">
+    <row r="235" ht="9.75" customHeight="1">
       <c r="A235" s="1"/>
       <c r="B235" s="1"/>
       <c r="C235" s="1"/>
@@ -3920,7 +4090,7 @@
       <c r="H235" s="1"/>
       <c r="I235" s="1"/>
     </row>
-    <row r="236" ht="9.75" customHeight="1" spans="1:9">
+    <row r="236" ht="9.75" customHeight="1">
       <c r="A236" s="1"/>
       <c r="B236" s="1"/>
       <c r="C236" s="1"/>
@@ -3931,7 +4101,7 @@
       <c r="H236" s="1"/>
       <c r="I236" s="1"/>
     </row>
-    <row r="237" ht="9.75" customHeight="1" spans="1:9">
+    <row r="237" ht="9.75" customHeight="1">
       <c r="A237" s="1"/>
       <c r="B237" s="1"/>
       <c r="C237" s="1"/>
@@ -3942,7 +4112,7 @@
       <c r="H237" s="1"/>
       <c r="I237" s="1"/>
     </row>
-    <row r="238" ht="9.75" customHeight="1" spans="1:9">
+    <row r="238" ht="9.75" customHeight="1">
       <c r="A238" s="1"/>
       <c r="B238" s="1"/>
       <c r="C238" s="1"/>
@@ -3953,7 +4123,7 @@
       <c r="H238" s="1"/>
       <c r="I238" s="1"/>
     </row>
-    <row r="239" ht="9.75" customHeight="1" spans="1:9">
+    <row r="239" ht="9.75" customHeight="1">
       <c r="A239" s="1"/>
       <c r="B239" s="1"/>
       <c r="C239" s="1"/>
@@ -4727,6 +4897,8 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B7:B40"/>
+    <mergeCell ref="C7:I9"/>
     <mergeCell ref="F10:I10"/>
     <mergeCell ref="C12:H12"/>
     <mergeCell ref="C13:H13"/>
@@ -4735,8 +4907,11 @@
     <mergeCell ref="D17:G17"/>
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="F19:H19"/>
+    <mergeCell ref="C20:H22"/>
     <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C24:H26"/>
     <mergeCell ref="D28:H28"/>
+    <mergeCell ref="C29:H30"/>
     <mergeCell ref="D32:H32"/>
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="F35:H35"/>
@@ -4744,14 +4919,10 @@
     <mergeCell ref="F36:H36"/>
     <mergeCell ref="D38:F38"/>
     <mergeCell ref="D39:F39"/>
-    <mergeCell ref="B7:B40"/>
-    <mergeCell ref="C20:H22"/>
-    <mergeCell ref="C24:H26"/>
-    <mergeCell ref="C29:H30"/>
-    <mergeCell ref="C7:I9"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
🐛 fix: fixed templates with missing data
</commit_message>
<xml_diff>
--- a/apps/excel-service/templates/NomadDocs/Cash Receipt Order.xlsx
+++ b/apps/excel-service/templates/NomadDocs/Cash Receipt Order.xlsx
@@ -53,7 +53,7 @@
     <t>{customer.fullnameClient}</t>
   </si>
   <si>
-    <t xml:space="preserve">{organization.organization}, {organization.address}</t>
+    <t xml:space="preserve">{organization.organization}, г.{organization.city}, {organization.index}, {organization.address}</t>
   </si>
   <si>
     <t xml:space="preserve">Основание: Договор               №{enumeration}               от  {documentDate.0}г </t>
@@ -105,10 +105,9 @@
     <numFmt numFmtId="166" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="167" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="27">
     <font>
       <sz val="8.000000"/>
-      <color indexed="64"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -258,11 +257,6 @@
       <sz val="8.000000"/>
       <color theme="1"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="8.000000"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -556,7 +550,7 @@
       <right style="none"/>
       <top style="none"/>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
     </border>
@@ -728,14 +722,14 @@
     <xf fontId="23" fillId="0" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="24" fillId="0" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="25" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="9" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="24" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="23" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="26" fillId="0" borderId="9" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="25" fillId="0" borderId="9" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="23" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -753,7 +747,7 @@
     <xf fontId="23" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="27" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="26" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf fontId="23" fillId="0" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -867,13 +861,13 @@
         <color theme="1"/>
       </font>
       <border>
-        <left/>
-        <right/>
+        <left style="none"/>
+        <right style="none"/>
         <top style="double">
           <color theme="4"/>
         </top>
-        <bottom/>
-        <diagonal/>
+        <bottom style="none"/>
+        <diagonal style="none"/>
       </border>
     </dxf>
     <dxf>
@@ -893,7 +887,7 @@
         <bottom style="thin">
           <color theme="4"/>
         </bottom>
-        <diagonal/>
+        <diagonal style="none"/>
         <horizontal style="thin">
           <color theme="4" tint="0.39997558519241899"/>
         </horizontal>
@@ -920,13 +914,13 @@
         <color theme="1"/>
       </font>
       <border>
-        <left/>
-        <right/>
-        <top/>
+        <left style="none"/>
+        <right style="none"/>
+        <top style="none"/>
         <bottom style="thin">
           <color theme="4" tint="0.39997558519241899"/>
         </bottom>
-        <diagonal/>
+        <diagonal style="none"/>
       </border>
     </dxf>
     <dxf>
@@ -935,15 +929,15 @@
         <color theme="1"/>
       </font>
       <border>
-        <left/>
-        <right/>
+        <left style="none"/>
+        <right style="none"/>
         <top style="thin">
           <color theme="4"/>
         </top>
         <bottom style="thin">
           <color theme="4"/>
         </bottom>
-        <diagonal/>
+        <diagonal style="none"/>
       </border>
     </dxf>
     <dxf>
@@ -958,13 +952,13 @@
         </patternFill>
       </fill>
       <border>
-        <left/>
-        <right/>
-        <top/>
+        <left style="none"/>
+        <right style="none"/>
+        <top style="none"/>
         <bottom style="thin">
           <color theme="4" tint="0.39997558519241899"/>
         </bottom>
-        <diagonal/>
+        <diagonal style="none"/>
       </border>
     </dxf>
     <dxf>
@@ -978,13 +972,13 @@
         </patternFill>
       </fill>
       <border>
-        <left/>
-        <right/>
-        <top/>
+        <left style="none"/>
+        <right style="none"/>
+        <top style="none"/>
         <bottom style="thin">
           <color theme="4" tint="0.39997558519241899"/>
         </bottom>
-        <diagonal/>
+        <diagonal style="none"/>
       </border>
     </dxf>
     <dxf>
@@ -995,13 +989,13 @@
         </patternFill>
       </fill>
       <border>
-        <left/>
-        <right/>
-        <top/>
+        <left style="none"/>
+        <right style="none"/>
+        <top style="none"/>
         <bottom style="thin">
           <color theme="4" tint="0.39997558519241899"/>
         </bottom>
-        <diagonal/>
+        <diagonal style="none"/>
       </border>
     </dxf>
     <dxf>
@@ -1027,15 +1021,15 @@
         </patternFill>
       </fill>
       <border>
-        <left/>
-        <right/>
+        <left style="none"/>
+        <right style="none"/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241899"/>
         </top>
         <bottom style="thin">
           <color theme="4" tint="0.39997558519241899"/>
         </bottom>
-        <diagonal/>
+        <diagonal style="none"/>
       </border>
     </dxf>
   </dxfs>

</xml_diff>

<commit_message>
🔧 chore: changed the type of costPerDay to numeric & optimized deploy pipline
</commit_message>
<xml_diff>
--- a/apps/excel-service/templates/NomadDocs/Cash Receipt Order.xlsx
+++ b/apps/excel-service/templates/NomadDocs/Cash Receipt Order.xlsx
@@ -65,10 +65,10 @@
     <t>Сумма</t>
   </si>
   <si>
-    <t xml:space="preserve">  {totalPrice}  тенге  00 тиын</t>
+    <t xml:space="preserve">  {totalCost}  тенге  00 тиын</t>
   </si>
   <si>
-    <t xml:space="preserve">{totalPriceWords} 00 тиын</t>
+    <t xml:space="preserve">{totalCostRu} 00 тиын</t>
   </si>
   <si>
     <t>прописью</t>

</xml_diff>

<commit_message>
✨ feat: added support float type for cost
</commit_message>
<xml_diff>
--- a/apps/excel-service/templates/NomadDocs/Cash Receipt Order.xlsx
+++ b/apps/excel-service/templates/NomadDocs/Cash Receipt Order.xlsx
@@ -65,10 +65,10 @@
     <t>Сумма</t>
   </si>
   <si>
-    <t xml:space="preserve">  {totalCost}  тенге  00 тиын</t>
+    <t xml:space="preserve">  {totalCost}  тенге  {totalCostCents} тиын</t>
   </si>
   <si>
-    <t xml:space="preserve">{totalCostRu} 00 тиын</t>
+    <t xml:space="preserve">{totalCostRu}{totalCostCentsRu} тиын</t>
   </si>
   <si>
     <t>прописью</t>

</xml_diff>